<commit_message>
Align CEE supplementary materials and document sampling and reproduction scope
</commit_message>
<xml_diff>
--- a/supplementary-materials/tables/Table_S06.xlsx
+++ b/supplementary-materials/tables/Table_S06.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S6" sheetId="1" r:id="Rf3124a0a9f13430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S6" sheetId="1" r:id="R52448b0600034483"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2711,14 +2711,18 @@
       <x:c r="F38" s="8" t="s">
         <x:v>222</x:v>
       </x:c>
-      <x:c r="G38" s="8" t="s">
-        <x:v>223</x:v>
+      <x:c r="G38" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">For H5, standardise weekly host opportunities separately and average. For HEQZ, use annual-mean opportunity, standardise groups separately, average and re-standardise.</x:t>
+        </x:is>
       </x:c>
       <x:c r="H38" s="8" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="I38" s="8" t="s">
-        <x:v>55</x:v>
+      <x:c r="I38" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Week (H5); annual mean (HEQZ)</x:t>
+        </x:is>
       </x:c>
       <x:c r="J38" s="8" t="s">
         <x:v>224</x:v>
@@ -2959,14 +2963,18 @@
       <x:c r="F45" s="8" t="s">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="G45" s="8" t="s">
-        <x:v>257</x:v>
+      <x:c r="G45" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Count predictor-wise range exceedances for each HEX.</x:t>
+        </x:is>
       </x:c>
       <x:c r="H45" s="8" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="I45" s="8" t="s">
-        <x:v>55</x:v>
+      <x:c r="I45" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Static; repeated across 52 weeks</x:t>
+        </x:is>
       </x:c>
       <x:c r="J45" s="8" t="s">
         <x:v>258</x:v>
@@ -2997,8 +3005,10 @@
       <x:c r="D46" s="9" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="E46" s="9" t="s">
-        <x:v>264</x:v>
+      <x:c r="E46" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Nearest distance from a city HEX to the training predictor space after scaling.</x:t>
+        </x:is>
       </x:c>
       <x:c r="F46" s="9" t="s">
         <x:v>256</x:v>
@@ -3009,8 +3019,10 @@
       <x:c r="H46" s="9" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="I46" s="9" t="s">
-        <x:v>55</x:v>
+      <x:c r="I46" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Static; repeated across 52 weeks</x:t>
+        </x:is>
       </x:c>
       <x:c r="J46" s="9" t="s">
         <x:v>266</x:v>
@@ -3051,8 +3063,10 @@
       <x:c r="H47" s="8" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="I47" s="8" t="s">
-        <x:v>55</x:v>
+      <x:c r="I47" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Static; repeated across 52 weeks</x:t>
+        </x:is>
       </x:c>
       <x:c r="J47" s="8" t="s">
         <x:v>250</x:v>
@@ -3093,8 +3107,10 @@
       <x:c r="H48" s="9" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="I48" s="9" t="s">
-        <x:v>280</x:v>
+      <x:c r="I48" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Static; repeated across 52 weeks</x:t>
+        </x:is>
       </x:c>
       <x:c r="J48" s="9" t="s">
         <x:v>250</x:v>
@@ -3123,14 +3139,18 @@
       <x:c r="D49" s="8" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="E49" s="8" t="s">
-        <x:v>287</x:v>
+      <x:c r="E49" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Expected count among 24 dawn samples on a reference day, averaged across W15–W21.</x:t>
+        </x:is>
       </x:c>
       <x:c r="F49" s="8" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="G49" s="8" t="s">
-        <x:v>289</x:v>
+      <x:c r="G49" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sum draw-wise probabilities over the 24 scheduled dawn samples, then average weekly counts across W15–W21.</x:t>
+        </x:is>
       </x:c>
       <x:c r="H49" s="8" t="s">
         <x:v>249</x:v>
@@ -3167,14 +3187,20 @@
       <x:c r="D50" s="9" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="E50" s="9" t="str">
-        <x:v>Posterior probability that the beta-binomial posterior predictive count for the declared dawn and seasonal window contains at least one Koel-positive sampled minute.</x:v>
-      </x:c>
-      <x:c r="F50" s="9" t="str">
-        <x:v>Posterior predictive beta-binomial count distribution</x:v>
-      </x:c>
-      <x:c r="G50" s="9" t="str">
-        <x:v>For each posterior draw, simulate the declared window from the fitted beta-binomial count process, record whether K_window ≥ 1, and summarise the indicator across draws.</x:v>
+      <x:c r="E50" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Probability of at least one positive sample among 24 dawn samples on a reference day, averaged across W15–W21.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F50" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Beta-binomial posterior predictive zero-count probabilities</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G50" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">For each draw, calculate window and full-day beta-binomial zero-count probabilities, condition on a positive day, combine with ψ and p, then average weekly probabilities across W15–W21.</x:t>
+        </x:is>
       </x:c>
       <x:c r="H50" s="9" t="s">
         <x:v>249</x:v>
@@ -3293,8 +3319,10 @@
       <x:c r="D53" s="10" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="E53" s="10" t="str">
-        <x:v>Within-layer 0–100 rank combining Coverage Expansion, Prediction Validation or planning-sensitive context under the declared layer.</x:v>
+      <x:c r="E53" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Within-layer 0–100 display score. The public-facing layer combines scientific priority with planning-sensitive context and does not select sites.</x:t>
+        </x:is>
       </x:c>
       <x:c r="F53" s="10" t="s">
         <x:v>318</x:v>
@@ -3314,11 +3342,15 @@
       <x:c r="K53" s="10" t="s">
         <x:v>322</x:v>
       </x:c>
-      <x:c r="L53" s="10" t="s">
-        <x:v>323</x:v>
-      </x:c>
-      <x:c r="M53" s="10" t="s">
-        <x:v>324</x:v>
+      <x:c r="L53" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scientific routes select sites; public-facing layer is display only</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M53" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Outside-pool cells are missing/grey; eligible cells may have a score of zero.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N53" s="10" t="s">
         <x:v>325</x:v>

</xml_diff>

<commit_message>
Align SA materials and share de-identified model inputs
</commit_message>
<xml_diff>
--- a/supplementary-materials/tables/Table_S06.xlsx
+++ b/supplementary-materials/tables/Table_S06.xlsx
@@ -679,7 +679,7 @@
     <x:t xml:space="preserve">Three host posterior surfaces</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Standardise each group, average the three values, then re-standardise.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">standardised index</x:t>
@@ -781,7 +781,7 @@
     <x:t xml:space="preserve">Training and city predictor matrices</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Count predictor-wise range exceedances for each HEX-week.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">count</x:t>
@@ -802,7 +802,7 @@
     <x:t xml:space="preserve">DI</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Nearest distance from a city HEX-week to the training predictor space after scaling.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Compute nearest training-space distance with the frozen AOA variables.</x:t>
@@ -850,7 +850,7 @@
     <x:t xml:space="preserve">Combine the two labels using the prespecified four-tier rule.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Week or summary</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Controls reporting emphasis</x:t>
@@ -871,13 +871,13 @@
     <x:t xml:space="preserve">dawn_w15_w21_expected_positive_sampled_minutes</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Expected number of Koel-positive sampled minutes in the declared dawn and seasonal window.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Posterior sampled-minute exposure</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Sum draw-wise sampled-minute probabilities over scheduled minute opportunities.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Declared seasonal × diel window</x:t>
@@ -979,10 +979,10 @@
     <x:t xml:space="preserve">Within-layer rank</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Future PAM site selection</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Zero outside the layer-specific eligibility set.</x:t>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Relative design priority, not predicted Koel exposure.</x:t>

</xml_diff>